<commit_message>
Consolidate similarity analysis into single end-to-end Python script and master Excel file
</commit_message>
<xml_diff>
--- a/similarity_analysis/complete_movie_pairwise_similarity_analysis.xlsx
+++ b/similarity_analysis/complete_movie_pairwise_similarity_analysis.xlsx
@@ -784,11 +784,11 @@
         <v>0.9295</v>
       </c>
       <c r="Y3" t="n">
-        <v>0.25</v>
+        <v>0.28</v>
       </c>
       <c r="Z3" t="inlineStr">
         <is>
-          <t>YES (Collided)</t>
+          <t>NO (Pruned)</t>
         </is>
       </c>
       <c r="AA3" t="inlineStr">
@@ -899,7 +899,7 @@
         <v>1</v>
       </c>
       <c r="Y4" t="n">
-        <v>0.01</v>
+        <v>0</v>
       </c>
       <c r="Z4" t="inlineStr">
         <is>
@@ -1014,7 +1014,7 @@
         <v>1</v>
       </c>
       <c r="Y5" t="n">
-        <v>0.14</v>
+        <v>0.17</v>
       </c>
       <c r="Z5" t="inlineStr">
         <is>
@@ -1129,7 +1129,7 @@
         <v>1</v>
       </c>
       <c r="Y6" t="n">
-        <v>0.09</v>
+        <v>0.08</v>
       </c>
       <c r="Z6" t="inlineStr">
         <is>
@@ -1244,7 +1244,7 @@
         <v>0.9782</v>
       </c>
       <c r="Y7" t="n">
-        <v>0.05</v>
+        <v>0.06</v>
       </c>
       <c r="Z7" t="inlineStr">
         <is>
@@ -1359,7 +1359,7 @@
         <v>0.9599</v>
       </c>
       <c r="Y8" t="n">
-        <v>0.03</v>
+        <v>0</v>
       </c>
       <c r="Z8" t="inlineStr">
         <is>
@@ -1474,7 +1474,7 @@
         <v>0.9373</v>
       </c>
       <c r="Y9" t="n">
-        <v>0.4</v>
+        <v>0.44</v>
       </c>
       <c r="Z9" t="inlineStr">
         <is>
@@ -1589,7 +1589,7 @@
         <v>1</v>
       </c>
       <c r="Y10" t="n">
-        <v>0.02</v>
+        <v>0</v>
       </c>
       <c r="Z10" t="inlineStr">
         <is>
@@ -1704,7 +1704,7 @@
         <v>0.8508</v>
       </c>
       <c r="Y11" t="n">
-        <v>0.05</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="Z11" t="inlineStr">
         <is>
@@ -1819,7 +1819,7 @@
         <v>1</v>
       </c>
       <c r="Y12" t="n">
-        <v>0.05</v>
+        <v>0.11</v>
       </c>
       <c r="Z12" t="inlineStr">
         <is>
@@ -1934,7 +1934,7 @@
         <v>1</v>
       </c>
       <c r="Y13" t="n">
-        <v>0.03</v>
+        <v>0</v>
       </c>
       <c r="Z13" t="inlineStr">
         <is>
@@ -2049,7 +2049,7 @@
         <v>1</v>
       </c>
       <c r="Y14" t="n">
-        <v>0.3</v>
+        <v>0.17</v>
       </c>
       <c r="Z14" t="inlineStr">
         <is>
@@ -2164,7 +2164,7 @@
         <v>1</v>
       </c>
       <c r="Y15" t="n">
-        <v>0.09</v>
+        <v>0.05</v>
       </c>
       <c r="Z15" t="inlineStr">
         <is>
@@ -2279,7 +2279,7 @@
         <v>0.9797</v>
       </c>
       <c r="Y16" t="n">
-        <v>0.22</v>
+        <v>0.16</v>
       </c>
       <c r="Z16" t="inlineStr">
         <is>
@@ -2509,7 +2509,7 @@
         <v>0.9696</v>
       </c>
       <c r="Y18" t="n">
-        <v>0.2</v>
+        <v>0.18</v>
       </c>
       <c r="Z18" t="inlineStr">
         <is>
@@ -2624,7 +2624,7 @@
         <v>0.981</v>
       </c>
       <c r="Y19" t="n">
-        <v>0.17</v>
+        <v>0.13</v>
       </c>
       <c r="Z19" t="inlineStr">
         <is>
@@ -2739,7 +2739,7 @@
         <v>0.9877</v>
       </c>
       <c r="Y20" t="n">
-        <v>0.06</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="Z20" t="inlineStr">
         <is>
@@ -2854,7 +2854,7 @@
         <v>0.9875</v>
       </c>
       <c r="Y21" t="n">
-        <v>0.06</v>
+        <v>0.02</v>
       </c>
       <c r="Z21" t="inlineStr">
         <is>
@@ -2969,7 +2969,7 @@
         <v>1</v>
       </c>
       <c r="Y22" t="n">
-        <v>0.03</v>
+        <v>0.09</v>
       </c>
       <c r="Z22" t="inlineStr">
         <is>
@@ -3084,7 +3084,7 @@
         <v>0.9544</v>
       </c>
       <c r="Y23" t="n">
-        <v>0.16</v>
+        <v>0.21</v>
       </c>
       <c r="Z23" t="inlineStr">
         <is>
@@ -3199,7 +3199,7 @@
         <v>1</v>
       </c>
       <c r="Y24" t="n">
-        <v>0.06</v>
+        <v>0.05</v>
       </c>
       <c r="Z24" t="inlineStr">
         <is>
@@ -3314,7 +3314,7 @@
         <v>0.9867</v>
       </c>
       <c r="Y25" t="n">
-        <v>0.29</v>
+        <v>0.24</v>
       </c>
       <c r="Z25" t="inlineStr">
         <is>
@@ -3429,11 +3429,11 @@
         <v>0.7571</v>
       </c>
       <c r="Y26" t="n">
-        <v>0.39</v>
+        <v>0.46</v>
       </c>
       <c r="Z26" t="inlineStr">
         <is>
-          <t>NO (Pruned)</t>
+          <t>YES (Collided)</t>
         </is>
       </c>
       <c r="AA26" t="inlineStr">
@@ -3544,7 +3544,7 @@
         <v>1</v>
       </c>
       <c r="Y27" t="n">
-        <v>0.08</v>
+        <v>0.02</v>
       </c>
       <c r="Z27" t="inlineStr">
         <is>
@@ -3659,7 +3659,7 @@
         <v>0.9098000000000001</v>
       </c>
       <c r="Y28" t="n">
-        <v>0.29</v>
+        <v>0.22</v>
       </c>
       <c r="Z28" t="inlineStr">
         <is>
@@ -3889,7 +3889,7 @@
         <v>0.9449</v>
       </c>
       <c r="Y30" t="n">
-        <v>0.2</v>
+        <v>0.27</v>
       </c>
       <c r="Z30" t="inlineStr">
         <is>
@@ -4004,7 +4004,7 @@
         <v>1</v>
       </c>
       <c r="Y31" t="n">
-        <v>0.11</v>
+        <v>0.04</v>
       </c>
       <c r="Z31" t="inlineStr">
         <is>
@@ -4119,7 +4119,7 @@
         <v>0.7345</v>
       </c>
       <c r="Y32" t="n">
-        <v>0.1</v>
+        <v>0.16</v>
       </c>
       <c r="Z32" t="inlineStr">
         <is>
@@ -4349,7 +4349,7 @@
         <v>0.8768</v>
       </c>
       <c r="Y34" t="n">
-        <v>0.39</v>
+        <v>0.32</v>
       </c>
       <c r="Z34" t="inlineStr">
         <is>
@@ -4464,7 +4464,7 @@
         <v>1</v>
       </c>
       <c r="Y35" t="n">
-        <v>0.03</v>
+        <v>0.12</v>
       </c>
       <c r="Z35" t="inlineStr">
         <is>
@@ -4579,7 +4579,7 @@
         <v>0.9728</v>
       </c>
       <c r="Y36" t="n">
-        <v>0.22</v>
+        <v>0.29</v>
       </c>
       <c r="Z36" t="inlineStr">
         <is>
@@ -4694,7 +4694,7 @@
         <v>1</v>
       </c>
       <c r="Y37" t="n">
-        <v>0.03</v>
+        <v>0.01</v>
       </c>
       <c r="Z37" t="inlineStr">
         <is>
@@ -4809,7 +4809,7 @@
         <v>0.9572000000000001</v>
       </c>
       <c r="Y38" t="n">
-        <v>0.26</v>
+        <v>0.32</v>
       </c>
       <c r="Z38" t="inlineStr">
         <is>
@@ -4924,7 +4924,7 @@
         <v>0.994</v>
       </c>
       <c r="Y39" t="n">
-        <v>0.06</v>
+        <v>0.05</v>
       </c>
       <c r="Z39" t="inlineStr">
         <is>
@@ -5039,7 +5039,7 @@
         <v>1</v>
       </c>
       <c r="Y40" t="n">
-        <v>0</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="Z40" t="inlineStr">
         <is>
@@ -5154,7 +5154,7 @@
         <v>0.9883999999999999</v>
       </c>
       <c r="Y41" t="n">
-        <v>0.16</v>
+        <v>0.15</v>
       </c>
       <c r="Z41" t="inlineStr">
         <is>
@@ -5269,7 +5269,7 @@
         <v>0.9196</v>
       </c>
       <c r="Y42" t="n">
-        <v>0.24</v>
+        <v>0.14</v>
       </c>
       <c r="Z42" t="inlineStr">
         <is>
@@ -5384,7 +5384,7 @@
         <v>0.8544</v>
       </c>
       <c r="Y43" t="n">
-        <v>0.28</v>
+        <v>0.33</v>
       </c>
       <c r="Z43" t="inlineStr">
         <is>
@@ -5499,7 +5499,7 @@
         <v>0.972</v>
       </c>
       <c r="Y44" t="n">
-        <v>0.19</v>
+        <v>0.26</v>
       </c>
       <c r="Z44" t="inlineStr">
         <is>
@@ -5614,7 +5614,7 @@
         <v>0.946</v>
       </c>
       <c r="Y45" t="n">
-        <v>0.43</v>
+        <v>0.4</v>
       </c>
       <c r="Z45" t="inlineStr">
         <is>
@@ -5959,7 +5959,7 @@
         <v>0.9496</v>
       </c>
       <c r="Y48" t="n">
-        <v>0.03</v>
+        <v>0.05</v>
       </c>
       <c r="Z48" t="inlineStr">
         <is>
@@ -6189,7 +6189,7 @@
         <v>0.9031</v>
       </c>
       <c r="Y50" t="n">
-        <v>0.22</v>
+        <v>0.3</v>
       </c>
       <c r="Z50" t="inlineStr">
         <is>
@@ -6304,7 +6304,7 @@
         <v>0.9674</v>
       </c>
       <c r="Y51" t="n">
-        <v>0.02</v>
+        <v>0.01</v>
       </c>
       <c r="Z51" t="inlineStr">
         <is>
@@ -6419,7 +6419,7 @@
         <v>0.97</v>
       </c>
       <c r="Y52" t="n">
-        <v>0.1</v>
+        <v>0.11</v>
       </c>
       <c r="Z52" t="inlineStr">
         <is>
@@ -6534,7 +6534,7 @@
         <v>0.9871</v>
       </c>
       <c r="Y53" t="n">
-        <v>0.2</v>
+        <v>0.16</v>
       </c>
       <c r="Z53" t="inlineStr">
         <is>
@@ -6649,7 +6649,7 @@
         <v>0.7585</v>
       </c>
       <c r="Y54" t="n">
-        <v>0.29</v>
+        <v>0.3</v>
       </c>
       <c r="Z54" t="inlineStr">
         <is>
@@ -6764,7 +6764,7 @@
         <v>0.9167</v>
       </c>
       <c r="Y55" t="n">
-        <v>0.24</v>
+        <v>0.18</v>
       </c>
       <c r="Z55" t="inlineStr">
         <is>
@@ -6879,7 +6879,7 @@
         <v>1</v>
       </c>
       <c r="Y56" t="n">
-        <v>0.03</v>
+        <v>0.08</v>
       </c>
       <c r="Z56" t="inlineStr">
         <is>
@@ -6994,7 +6994,7 @@
         <v>0.9859</v>
       </c>
       <c r="Y57" t="n">
-        <v>0.1</v>
+        <v>0.11</v>
       </c>
       <c r="Z57" t="inlineStr">
         <is>
@@ -7109,7 +7109,7 @@
         <v>0.9067</v>
       </c>
       <c r="Y58" t="n">
-        <v>0.39</v>
+        <v>0.25</v>
       </c>
       <c r="Z58" t="inlineStr">
         <is>
@@ -7224,7 +7224,7 @@
         <v>0.9869</v>
       </c>
       <c r="Y59" t="n">
-        <v>0.19</v>
+        <v>0.15</v>
       </c>
       <c r="Z59" t="inlineStr">
         <is>
@@ -7454,7 +7454,7 @@
         <v>1</v>
       </c>
       <c r="Y61" t="n">
-        <v>0.11</v>
+        <v>0.06</v>
       </c>
       <c r="Z61" t="inlineStr">
         <is>
@@ -7569,7 +7569,7 @@
         <v>0.9415</v>
       </c>
       <c r="Y62" t="n">
-        <v>0.21</v>
+        <v>0.12</v>
       </c>
       <c r="Z62" t="inlineStr">
         <is>
@@ -7684,7 +7684,7 @@
         <v>0.9391</v>
       </c>
       <c r="Y63" t="n">
-        <v>0</v>
+        <v>0.02</v>
       </c>
       <c r="Z63" t="inlineStr">
         <is>
@@ -7799,11 +7799,11 @@
         <v>0.851</v>
       </c>
       <c r="Y64" t="n">
-        <v>0.43</v>
+        <v>0.4</v>
       </c>
       <c r="Z64" t="inlineStr">
         <is>
-          <t>YES (Collided)</t>
+          <t>NO (Pruned)</t>
         </is>
       </c>
       <c r="AA64" t="inlineStr">
@@ -7914,7 +7914,7 @@
         <v>0.9946</v>
       </c>
       <c r="Y65" t="n">
-        <v>0.13</v>
+        <v>0.15</v>
       </c>
       <c r="Z65" t="inlineStr">
         <is>
@@ -8029,7 +8029,7 @@
         <v>1</v>
       </c>
       <c r="Y66" t="n">
-        <v>0.04</v>
+        <v>0.08</v>
       </c>
       <c r="Z66" t="inlineStr">
         <is>
@@ -8144,7 +8144,7 @@
         <v>0.9871</v>
       </c>
       <c r="Y67" t="n">
-        <v>0.08</v>
+        <v>0.04</v>
       </c>
       <c r="Z67" t="inlineStr">
         <is>
@@ -8259,7 +8259,7 @@
         <v>0.9297</v>
       </c>
       <c r="Y68" t="n">
-        <v>0.17</v>
+        <v>0.12</v>
       </c>
       <c r="Z68" t="inlineStr">
         <is>
@@ -8374,7 +8374,7 @@
         <v>0.919</v>
       </c>
       <c r="Y69" t="n">
-        <v>0.32</v>
+        <v>0.24</v>
       </c>
       <c r="Z69" t="inlineStr">
         <is>
@@ -8489,7 +8489,7 @@
         <v>0.9693000000000001</v>
       </c>
       <c r="Y70" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.05</v>
       </c>
       <c r="Z70" t="inlineStr">
         <is>
@@ -8604,7 +8604,7 @@
         <v>0.9361</v>
       </c>
       <c r="Y71" t="n">
-        <v>0.2</v>
+        <v>0.19</v>
       </c>
       <c r="Z71" t="inlineStr">
         <is>
@@ -8719,7 +8719,7 @@
         <v>0.9651999999999999</v>
       </c>
       <c r="Y72" t="n">
-        <v>0.1</v>
+        <v>0.04</v>
       </c>
       <c r="Z72" t="inlineStr">
         <is>
@@ -8834,7 +8834,7 @@
         <v>1</v>
       </c>
       <c r="Y73" t="n">
-        <v>0.06</v>
+        <v>0.1</v>
       </c>
       <c r="Z73" t="inlineStr">
         <is>
@@ -8949,7 +8949,7 @@
         <v>0.9494</v>
       </c>
       <c r="Y74" t="n">
-        <v>0.08</v>
+        <v>0.06</v>
       </c>
       <c r="Z74" t="inlineStr">
         <is>
@@ -9064,7 +9064,7 @@
         <v>1</v>
       </c>
       <c r="Y75" t="n">
-        <v>0.05</v>
+        <v>0.03</v>
       </c>
       <c r="Z75" t="inlineStr">
         <is>
@@ -9179,7 +9179,7 @@
         <v>1</v>
       </c>
       <c r="Y76" t="n">
-        <v>0.02</v>
+        <v>0.01</v>
       </c>
       <c r="Z76" t="inlineStr">
         <is>
@@ -9294,7 +9294,7 @@
         <v>0.9368</v>
       </c>
       <c r="Y77" t="n">
-        <v>0.09</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="Z77" t="inlineStr">
         <is>
@@ -9409,7 +9409,7 @@
         <v>0.9320000000000001</v>
       </c>
       <c r="Y78" t="n">
-        <v>0.34</v>
+        <v>0.29</v>
       </c>
       <c r="Z78" t="inlineStr">
         <is>
@@ -9524,7 +9524,7 @@
         <v>1</v>
       </c>
       <c r="Y79" t="n">
-        <v>0.05</v>
+        <v>0.1</v>
       </c>
       <c r="Z79" t="inlineStr">
         <is>
@@ -9639,7 +9639,7 @@
         <v>0.9731</v>
       </c>
       <c r="Y80" t="n">
-        <v>0.04</v>
+        <v>0.02</v>
       </c>
       <c r="Z80" t="inlineStr">
         <is>
@@ -9869,7 +9869,7 @@
         <v>0.9784</v>
       </c>
       <c r="Y82" t="n">
-        <v>0.41</v>
+        <v>0.3</v>
       </c>
       <c r="Z82" t="inlineStr">
         <is>
@@ -9984,7 +9984,7 @@
         <v>1</v>
       </c>
       <c r="Y83" t="n">
-        <v>0.02</v>
+        <v>0.03</v>
       </c>
       <c r="Z83" t="inlineStr">
         <is>
@@ -10099,7 +10099,7 @@
         <v>0.864</v>
       </c>
       <c r="Y84" t="n">
-        <v>0.19</v>
+        <v>0.17</v>
       </c>
       <c r="Z84" t="inlineStr">
         <is>
@@ -10214,7 +10214,7 @@
         <v>0.9419999999999999</v>
       </c>
       <c r="Y85" t="n">
-        <v>0.02</v>
+        <v>0.01</v>
       </c>
       <c r="Z85" t="inlineStr">
         <is>
@@ -10329,7 +10329,7 @@
         <v>0.9104</v>
       </c>
       <c r="Y86" t="n">
-        <v>0.22</v>
+        <v>0.16</v>
       </c>
       <c r="Z86" t="inlineStr">
         <is>
@@ -10444,7 +10444,7 @@
         <v>0.9684</v>
       </c>
       <c r="Y87" t="n">
-        <v>0.13</v>
+        <v>0.14</v>
       </c>
       <c r="Z87" t="inlineStr">
         <is>
@@ -10559,7 +10559,7 @@
         <v>0.8813</v>
       </c>
       <c r="Y88" t="n">
-        <v>0.12</v>
+        <v>0.11</v>
       </c>
       <c r="Z88" t="inlineStr">
         <is>
@@ -10674,7 +10674,7 @@
         <v>0.8908</v>
       </c>
       <c r="Y89" t="n">
-        <v>0.14</v>
+        <v>0.13</v>
       </c>
       <c r="Z89" t="inlineStr">
         <is>
@@ -10789,7 +10789,7 @@
         <v>0.895</v>
       </c>
       <c r="Y90" t="n">
-        <v>0.31</v>
+        <v>0.24</v>
       </c>
       <c r="Z90" t="inlineStr">
         <is>
@@ -10904,7 +10904,7 @@
         <v>1</v>
       </c>
       <c r="Y91" t="n">
-        <v>0.03</v>
+        <v>0.05</v>
       </c>
       <c r="Z91" t="inlineStr">
         <is>
@@ -11019,7 +11019,7 @@
         <v>1</v>
       </c>
       <c r="Y92" t="n">
-        <v>0.12</v>
+        <v>0.08</v>
       </c>
       <c r="Z92" t="inlineStr">
         <is>
@@ -11134,7 +11134,7 @@
         <v>1</v>
       </c>
       <c r="Y93" t="n">
-        <v>0.06</v>
+        <v>0.05</v>
       </c>
       <c r="Z93" t="inlineStr">
         <is>
@@ -11249,7 +11249,7 @@
         <v>0.9703000000000001</v>
       </c>
       <c r="Y94" t="n">
-        <v>0.11</v>
+        <v>0.06</v>
       </c>
       <c r="Z94" t="inlineStr">
         <is>
@@ -11364,7 +11364,7 @@
         <v>1</v>
       </c>
       <c r="Y95" t="n">
-        <v>0.02</v>
+        <v>0</v>
       </c>
       <c r="Z95" t="inlineStr">
         <is>
@@ -11479,7 +11479,7 @@
         <v>0.9699</v>
       </c>
       <c r="Y96" t="n">
-        <v>0.14</v>
+        <v>0.13</v>
       </c>
       <c r="Z96" t="inlineStr">
         <is>
@@ -11709,7 +11709,7 @@
         <v>0.9612000000000001</v>
       </c>
       <c r="Y98" t="n">
-        <v>0.05</v>
+        <v>0.03</v>
       </c>
       <c r="Z98" t="inlineStr">
         <is>
@@ -11824,7 +11824,7 @@
         <v>0.9824000000000001</v>
       </c>
       <c r="Y99" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.12</v>
       </c>
       <c r="Z99" t="inlineStr">
         <is>
@@ -11939,7 +11939,7 @@
         <v>0.9516</v>
       </c>
       <c r="Y100" t="n">
-        <v>0.17</v>
+        <v>0.08</v>
       </c>
       <c r="Z100" t="inlineStr">
         <is>
@@ -12054,7 +12054,7 @@
         <v>0.9034</v>
       </c>
       <c r="Y101" t="n">
-        <v>0.22</v>
+        <v>0.17</v>
       </c>
       <c r="Z101" t="inlineStr">
         <is>
@@ -12169,7 +12169,7 @@
         <v>1</v>
       </c>
       <c r="Y102" t="n">
-        <v>0.03</v>
+        <v>0.01</v>
       </c>
       <c r="Z102" t="inlineStr">
         <is>
@@ -12284,7 +12284,7 @@
         <v>0.9554</v>
       </c>
       <c r="Y103" t="n">
-        <v>0.08</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="Z103" t="inlineStr">
         <is>
@@ -12514,7 +12514,7 @@
         <v>0.9035</v>
       </c>
       <c r="Y105" t="n">
-        <v>0.04</v>
+        <v>0.01</v>
       </c>
       <c r="Z105" t="inlineStr">
         <is>
@@ -12629,7 +12629,7 @@
         <v>0.8697</v>
       </c>
       <c r="Y106" t="n">
-        <v>0.27</v>
+        <v>0.2</v>
       </c>
       <c r="Z106" t="inlineStr">
         <is>
@@ -12744,7 +12744,7 @@
         <v>0.8582</v>
       </c>
       <c r="Y107" t="n">
-        <v>0.08</v>
+        <v>0.05</v>
       </c>
       <c r="Z107" t="inlineStr">
         <is>
@@ -12859,7 +12859,7 @@
         <v>1</v>
       </c>
       <c r="Y108" t="n">
-        <v>0.05</v>
+        <v>0.08</v>
       </c>
       <c r="Z108" t="inlineStr">
         <is>
@@ -13204,7 +13204,7 @@
         <v>1</v>
       </c>
       <c r="Y111" t="n">
-        <v>0.06</v>
+        <v>0.04</v>
       </c>
       <c r="Z111" t="inlineStr">
         <is>
@@ -13319,7 +13319,7 @@
         <v>0.9801</v>
       </c>
       <c r="Y112" t="n">
-        <v>0.13</v>
+        <v>0.16</v>
       </c>
       <c r="Z112" t="inlineStr">
         <is>
@@ -13549,7 +13549,7 @@
         <v>1</v>
       </c>
       <c r="Y114" t="n">
-        <v>0.03</v>
+        <v>0.01</v>
       </c>
       <c r="Z114" t="inlineStr">
         <is>
@@ -13664,7 +13664,7 @@
         <v>0.9848</v>
       </c>
       <c r="Y115" t="n">
-        <v>0.25</v>
+        <v>0.24</v>
       </c>
       <c r="Z115" t="inlineStr">
         <is>
@@ -13779,7 +13779,7 @@
         <v>0.9678</v>
       </c>
       <c r="Y116" t="n">
-        <v>0.24</v>
+        <v>0.26</v>
       </c>
       <c r="Z116" t="inlineStr">
         <is>
@@ -13894,7 +13894,7 @@
         <v>0.9467</v>
       </c>
       <c r="Y117" t="n">
-        <v>0.25</v>
+        <v>0.19</v>
       </c>
       <c r="Z117" t="inlineStr">
         <is>
@@ -14124,7 +14124,7 @@
         <v>1</v>
       </c>
       <c r="Y119" t="n">
-        <v>0</v>
+        <v>0.02</v>
       </c>
       <c r="Z119" t="inlineStr">
         <is>
@@ -14239,7 +14239,7 @@
         <v>1</v>
       </c>
       <c r="Y120" t="n">
-        <v>0.03</v>
+        <v>0.04</v>
       </c>
       <c r="Z120" t="inlineStr">
         <is>
@@ -14354,7 +14354,7 @@
         <v>1</v>
       </c>
       <c r="Y121" t="n">
-        <v>0.04</v>
+        <v>0.01</v>
       </c>
       <c r="Z121" t="inlineStr">
         <is>
@@ -14469,7 +14469,7 @@
         <v>0.895</v>
       </c>
       <c r="Y122" t="n">
-        <v>0.29</v>
+        <v>0.21</v>
       </c>
       <c r="Z122" t="inlineStr">
         <is>
@@ -14584,7 +14584,7 @@
         <v>0.9533</v>
       </c>
       <c r="Y123" t="n">
-        <v>0.09</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="Z123" t="inlineStr">
         <is>
@@ -14699,7 +14699,7 @@
         <v>0.9696</v>
       </c>
       <c r="Y124" t="n">
-        <v>0.02</v>
+        <v>0.04</v>
       </c>
       <c r="Z124" t="inlineStr">
         <is>
@@ -14929,7 +14929,7 @@
         <v>0.9523</v>
       </c>
       <c r="Y126" t="n">
-        <v>0.16</v>
+        <v>0.12</v>
       </c>
       <c r="Z126" t="inlineStr">
         <is>
@@ -15159,7 +15159,7 @@
         <v>1</v>
       </c>
       <c r="Y128" t="n">
-        <v>0.01</v>
+        <v>0</v>
       </c>
       <c r="Z128" t="inlineStr">
         <is>
@@ -15504,7 +15504,7 @@
         <v>0.9785</v>
       </c>
       <c r="Y131" t="n">
-        <v>0.14</v>
+        <v>0.13</v>
       </c>
       <c r="Z131" t="inlineStr">
         <is>
@@ -15619,7 +15619,7 @@
         <v>0.954</v>
       </c>
       <c r="Y132" t="n">
-        <v>0.03</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="Z132" t="inlineStr">
         <is>
@@ -15734,7 +15734,7 @@
         <v>0.9354</v>
       </c>
       <c r="Y133" t="n">
-        <v>0.06</v>
+        <v>0.08</v>
       </c>
       <c r="Z133" t="inlineStr">
         <is>
@@ -15849,7 +15849,7 @@
         <v>1</v>
       </c>
       <c r="Y134" t="n">
-        <v>0.04</v>
+        <v>0.03</v>
       </c>
       <c r="Z134" t="inlineStr">
         <is>
@@ -16194,7 +16194,7 @@
         <v>0.9694</v>
       </c>
       <c r="Y137" t="n">
-        <v>0.14</v>
+        <v>0.18</v>
       </c>
       <c r="Z137" t="inlineStr">
         <is>
@@ -16309,7 +16309,7 @@
         <v>0.8774</v>
       </c>
       <c r="Y138" t="n">
-        <v>0.13</v>
+        <v>0.12</v>
       </c>
       <c r="Z138" t="inlineStr">
         <is>
@@ -16424,7 +16424,7 @@
         <v>0.9896</v>
       </c>
       <c r="Y139" t="n">
-        <v>0.29</v>
+        <v>0.32</v>
       </c>
       <c r="Z139" t="inlineStr">
         <is>
@@ -16539,7 +16539,7 @@
         <v>1</v>
       </c>
       <c r="Y140" t="n">
-        <v>0</v>
+        <v>0.02</v>
       </c>
       <c r="Z140" t="inlineStr">
         <is>
@@ -16884,7 +16884,7 @@
         <v>0.9796</v>
       </c>
       <c r="Y143" t="n">
-        <v>0.13</v>
+        <v>0.08</v>
       </c>
       <c r="Z143" t="inlineStr">
         <is>
@@ -16999,7 +16999,7 @@
         <v>1</v>
       </c>
       <c r="Y144" t="n">
-        <v>0.01</v>
+        <v>0.05</v>
       </c>
       <c r="Z144" t="inlineStr">
         <is>
@@ -17344,7 +17344,7 @@
         <v>0.983</v>
       </c>
       <c r="Y147" t="n">
-        <v>0.19</v>
+        <v>0.17</v>
       </c>
       <c r="Z147" t="inlineStr">
         <is>
@@ -17459,7 +17459,7 @@
         <v>1</v>
       </c>
       <c r="Y148" t="n">
-        <v>0.03</v>
+        <v>0.05</v>
       </c>
       <c r="Z148" t="inlineStr">
         <is>
@@ -17574,7 +17574,7 @@
         <v>0.99</v>
       </c>
       <c r="Y149" t="n">
-        <v>0.1</v>
+        <v>0.08</v>
       </c>
       <c r="Z149" t="inlineStr">
         <is>
@@ -17689,7 +17689,7 @@
         <v>1</v>
       </c>
       <c r="Y150" t="n">
-        <v>0.13</v>
+        <v>0.1</v>
       </c>
       <c r="Z150" t="inlineStr">
         <is>
@@ -17804,7 +17804,7 @@
         <v>0.9796</v>
       </c>
       <c r="Y151" t="n">
-        <v>0.21</v>
+        <v>0.19</v>
       </c>
       <c r="Z151" t="inlineStr">
         <is>
@@ -17919,7 +17919,7 @@
         <v>0.9752999999999999</v>
       </c>
       <c r="Y152" t="n">
-        <v>0.1</v>
+        <v>0.04</v>
       </c>
       <c r="Z152" t="inlineStr">
         <is>
@@ -18034,7 +18034,7 @@
         <v>1</v>
       </c>
       <c r="Y153" t="n">
-        <v>0.03</v>
+        <v>0.02</v>
       </c>
       <c r="Z153" t="inlineStr">
         <is>
@@ -18149,7 +18149,7 @@
         <v>0.8913</v>
       </c>
       <c r="Y154" t="n">
-        <v>0.23</v>
+        <v>0.25</v>
       </c>
       <c r="Z154" t="inlineStr">
         <is>
@@ -18264,7 +18264,7 @@
         <v>0.9288999999999999</v>
       </c>
       <c r="Y155" t="n">
-        <v>0.18</v>
+        <v>0.16</v>
       </c>
       <c r="Z155" t="inlineStr">
         <is>
@@ -18379,7 +18379,7 @@
         <v>0.9363</v>
       </c>
       <c r="Y156" t="n">
-        <v>0.28</v>
+        <v>0.24</v>
       </c>
       <c r="Z156" t="inlineStr">
         <is>
@@ -18494,7 +18494,7 @@
         <v>0.9396</v>
       </c>
       <c r="Y157" t="n">
-        <v>0.13</v>
+        <v>0.18</v>
       </c>
       <c r="Z157" t="inlineStr">
         <is>
@@ -18609,7 +18609,7 @@
         <v>1</v>
       </c>
       <c r="Y158" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.03</v>
       </c>
       <c r="Z158" t="inlineStr">
         <is>
@@ -18724,7 +18724,7 @@
         <v>0.9529</v>
       </c>
       <c r="Y159" t="n">
-        <v>0.11</v>
+        <v>0.14</v>
       </c>
       <c r="Z159" t="inlineStr">
         <is>
@@ -18839,7 +18839,7 @@
         <v>1</v>
       </c>
       <c r="Y160" t="n">
-        <v>0.09</v>
+        <v>0.12</v>
       </c>
       <c r="Z160" t="inlineStr">
         <is>
@@ -19069,7 +19069,7 @@
         <v>0.9963</v>
       </c>
       <c r="Y162" t="n">
-        <v>0.13</v>
+        <v>0.06</v>
       </c>
       <c r="Z162" t="inlineStr">
         <is>
@@ -19184,7 +19184,7 @@
         <v>0.893</v>
       </c>
       <c r="Y163" t="n">
-        <v>0.41</v>
+        <v>0.36</v>
       </c>
       <c r="Z163" t="inlineStr">
         <is>
@@ -19299,7 +19299,7 @@
         <v>0.9827</v>
       </c>
       <c r="Y164" t="n">
-        <v>0.02</v>
+        <v>0.03</v>
       </c>
       <c r="Z164" t="inlineStr">
         <is>
@@ -19414,7 +19414,7 @@
         <v>0.9594</v>
       </c>
       <c r="Y165" t="n">
-        <v>0.13</v>
+        <v>0.16</v>
       </c>
       <c r="Z165" t="inlineStr">
         <is>
@@ -19529,7 +19529,7 @@
         <v>1</v>
       </c>
       <c r="Y166" t="n">
-        <v>0.03</v>
+        <v>0</v>
       </c>
       <c r="Z166" t="inlineStr">
         <is>
@@ -19644,7 +19644,7 @@
         <v>0.9528</v>
       </c>
       <c r="Y167" t="n">
-        <v>0.19</v>
+        <v>0.23</v>
       </c>
       <c r="Z167" t="inlineStr">
         <is>
@@ -19759,7 +19759,7 @@
         <v>0.9532</v>
       </c>
       <c r="Y168" t="n">
-        <v>0.29</v>
+        <v>0.22</v>
       </c>
       <c r="Z168" t="inlineStr">
         <is>
@@ -20104,7 +20104,7 @@
         <v>0.9718</v>
       </c>
       <c r="Y171" t="n">
-        <v>0.13</v>
+        <v>0.09</v>
       </c>
       <c r="Z171" t="inlineStr">
         <is>
@@ -20219,7 +20219,7 @@
         <v>0.977</v>
       </c>
       <c r="Y172" t="n">
-        <v>0.14</v>
+        <v>0.13</v>
       </c>
       <c r="Z172" t="inlineStr">
         <is>
@@ -20334,7 +20334,7 @@
         <v>0.9283</v>
       </c>
       <c r="Y173" t="n">
-        <v>0.33</v>
+        <v>0.23</v>
       </c>
       <c r="Z173" t="inlineStr">
         <is>
@@ -20449,7 +20449,7 @@
         <v>0.9659</v>
       </c>
       <c r="Y174" t="n">
-        <v>0.22</v>
+        <v>0.18</v>
       </c>
       <c r="Z174" t="inlineStr">
         <is>
@@ -20564,11 +20564,11 @@
         <v>0.6267</v>
       </c>
       <c r="Y175" t="n">
-        <v>0.46</v>
+        <v>0.39</v>
       </c>
       <c r="Z175" t="inlineStr">
         <is>
-          <t>YES (Collided)</t>
+          <t>NO (Pruned)</t>
         </is>
       </c>
       <c r="AA175" t="inlineStr">
@@ -20679,7 +20679,7 @@
         <v>0.9816</v>
       </c>
       <c r="Y176" t="n">
-        <v>0.11</v>
+        <v>0.13</v>
       </c>
       <c r="Z176" t="inlineStr">
         <is>
@@ -20794,7 +20794,7 @@
         <v>0.9775</v>
       </c>
       <c r="Y177" t="n">
-        <v>0.13</v>
+        <v>0.09</v>
       </c>
       <c r="Z177" t="inlineStr">
         <is>
@@ -20909,7 +20909,7 @@
         <v>1</v>
       </c>
       <c r="Y178" t="n">
-        <v>0.03</v>
+        <v>0.05</v>
       </c>
       <c r="Z178" t="inlineStr">
         <is>
@@ -21024,7 +21024,7 @@
         <v>0.9826</v>
       </c>
       <c r="Y179" t="n">
-        <v>0.06</v>
+        <v>0.05</v>
       </c>
       <c r="Z179" t="inlineStr">
         <is>
@@ -21139,7 +21139,7 @@
         <v>1</v>
       </c>
       <c r="Y180" t="n">
-        <v>0.11</v>
+        <v>0.05</v>
       </c>
       <c r="Z180" t="inlineStr">
         <is>
@@ -21254,7 +21254,7 @@
         <v>1</v>
       </c>
       <c r="Y181" t="n">
-        <v>0.13</v>
+        <v>0.14</v>
       </c>
       <c r="Z181" t="inlineStr">
         <is>
@@ -21369,7 +21369,7 @@
         <v>0.9881</v>
       </c>
       <c r="Y182" t="n">
-        <v>0.23</v>
+        <v>0.16</v>
       </c>
       <c r="Z182" t="inlineStr">
         <is>
@@ -21599,7 +21599,7 @@
         <v>0.8469</v>
       </c>
       <c r="Y184" t="n">
-        <v>0.25</v>
+        <v>0.27</v>
       </c>
       <c r="Z184" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Sort Excel master sheet by movie_name, review_1_date, review_2_date
</commit_message>
<xml_diff>
--- a/similarity_analysis/complete_movie_pairwise_similarity_analysis.xlsx
+++ b/similarity_analysis/complete_movie_pairwise_similarity_analysis.xlsx
@@ -784,7 +784,7 @@
         <v>0.9295</v>
       </c>
       <c r="Y3" t="n">
-        <v>0.28</v>
+        <v>0.13</v>
       </c>
       <c r="Z3" t="inlineStr">
         <is>
@@ -899,7 +899,7 @@
         <v>1</v>
       </c>
       <c r="Y4" t="n">
-        <v>0</v>
+        <v>0.01</v>
       </c>
       <c r="Z4" t="inlineStr">
         <is>
@@ -1014,7 +1014,7 @@
         <v>1</v>
       </c>
       <c r="Y5" t="n">
-        <v>0.17</v>
+        <v>0.13</v>
       </c>
       <c r="Z5" t="inlineStr">
         <is>
@@ -1359,7 +1359,7 @@
         <v>0.9599</v>
       </c>
       <c r="Y8" t="n">
-        <v>0</v>
+        <v>0.05</v>
       </c>
       <c r="Z8" t="inlineStr">
         <is>
@@ -1474,7 +1474,7 @@
         <v>0.9373</v>
       </c>
       <c r="Y9" t="n">
-        <v>0.44</v>
+        <v>0.36</v>
       </c>
       <c r="Z9" t="inlineStr">
         <is>
@@ -1704,7 +1704,7 @@
         <v>0.8508</v>
       </c>
       <c r="Y11" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.08</v>
       </c>
       <c r="Z11" t="inlineStr">
         <is>
@@ -1819,7 +1819,7 @@
         <v>1</v>
       </c>
       <c r="Y12" t="n">
-        <v>0.11</v>
+        <v>0.06</v>
       </c>
       <c r="Z12" t="inlineStr">
         <is>
@@ -1934,7 +1934,7 @@
         <v>1</v>
       </c>
       <c r="Y13" t="n">
-        <v>0</v>
+        <v>0.01</v>
       </c>
       <c r="Z13" t="inlineStr">
         <is>
@@ -2049,7 +2049,7 @@
         <v>1</v>
       </c>
       <c r="Y14" t="n">
-        <v>0.17</v>
+        <v>0.18</v>
       </c>
       <c r="Z14" t="inlineStr">
         <is>
@@ -2164,7 +2164,7 @@
         <v>1</v>
       </c>
       <c r="Y15" t="n">
-        <v>0.05</v>
+        <v>0.08</v>
       </c>
       <c r="Z15" t="inlineStr">
         <is>
@@ -2279,7 +2279,7 @@
         <v>0.9797</v>
       </c>
       <c r="Y16" t="n">
-        <v>0.16</v>
+        <v>0.11</v>
       </c>
       <c r="Z16" t="inlineStr">
         <is>
@@ -2509,7 +2509,7 @@
         <v>0.9696</v>
       </c>
       <c r="Y18" t="n">
-        <v>0.18</v>
+        <v>0.14</v>
       </c>
       <c r="Z18" t="inlineStr">
         <is>
@@ -2624,7 +2624,7 @@
         <v>0.981</v>
       </c>
       <c r="Y19" t="n">
-        <v>0.13</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="Z19" t="inlineStr">
         <is>
@@ -2739,7 +2739,7 @@
         <v>0.9877</v>
       </c>
       <c r="Y20" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.1</v>
       </c>
       <c r="Z20" t="inlineStr">
         <is>
@@ -2854,7 +2854,7 @@
         <v>0.9875</v>
       </c>
       <c r="Y21" t="n">
-        <v>0.02</v>
+        <v>0.03</v>
       </c>
       <c r="Z21" t="inlineStr">
         <is>
@@ -2969,7 +2969,7 @@
         <v>1</v>
       </c>
       <c r="Y22" t="n">
-        <v>0.09</v>
+        <v>0.11</v>
       </c>
       <c r="Z22" t="inlineStr">
         <is>
@@ -3084,7 +3084,7 @@
         <v>0.9544</v>
       </c>
       <c r="Y23" t="n">
-        <v>0.21</v>
+        <v>0.17</v>
       </c>
       <c r="Z23" t="inlineStr">
         <is>
@@ -3199,7 +3199,7 @@
         <v>1</v>
       </c>
       <c r="Y24" t="n">
-        <v>0.05</v>
+        <v>0.02</v>
       </c>
       <c r="Z24" t="inlineStr">
         <is>
@@ -3314,7 +3314,7 @@
         <v>0.9867</v>
       </c>
       <c r="Y25" t="n">
-        <v>0.24</v>
+        <v>0.18</v>
       </c>
       <c r="Z25" t="inlineStr">
         <is>
@@ -3429,11 +3429,11 @@
         <v>0.7571</v>
       </c>
       <c r="Y26" t="n">
-        <v>0.46</v>
+        <v>0.29</v>
       </c>
       <c r="Z26" t="inlineStr">
         <is>
-          <t>YES (Collided)</t>
+          <t>NO (Pruned)</t>
         </is>
       </c>
       <c r="AA26" t="inlineStr">
@@ -3659,7 +3659,7 @@
         <v>0.9098000000000001</v>
       </c>
       <c r="Y28" t="n">
-        <v>0.22</v>
+        <v>0.24</v>
       </c>
       <c r="Z28" t="inlineStr">
         <is>
@@ -3889,7 +3889,7 @@
         <v>0.9449</v>
       </c>
       <c r="Y30" t="n">
-        <v>0.27</v>
+        <v>0.17</v>
       </c>
       <c r="Z30" t="inlineStr">
         <is>
@@ -4004,7 +4004,7 @@
         <v>1</v>
       </c>
       <c r="Y31" t="n">
-        <v>0.04</v>
+        <v>0.06</v>
       </c>
       <c r="Z31" t="inlineStr">
         <is>
@@ -4119,7 +4119,7 @@
         <v>0.7345</v>
       </c>
       <c r="Y32" t="n">
-        <v>0.16</v>
+        <v>0.15</v>
       </c>
       <c r="Z32" t="inlineStr">
         <is>
@@ -4234,7 +4234,7 @@
         <v>1</v>
       </c>
       <c r="Y33" t="n">
-        <v>0.05</v>
+        <v>0.08</v>
       </c>
       <c r="Z33" t="inlineStr">
         <is>
@@ -4349,7 +4349,7 @@
         <v>0.8768</v>
       </c>
       <c r="Y34" t="n">
-        <v>0.32</v>
+        <v>0.43</v>
       </c>
       <c r="Z34" t="inlineStr">
         <is>
@@ -4464,7 +4464,7 @@
         <v>1</v>
       </c>
       <c r="Y35" t="n">
-        <v>0.12</v>
+        <v>0.05</v>
       </c>
       <c r="Z35" t="inlineStr">
         <is>
@@ -4579,7 +4579,7 @@
         <v>0.9728</v>
       </c>
       <c r="Y36" t="n">
-        <v>0.29</v>
+        <v>0.23</v>
       </c>
       <c r="Z36" t="inlineStr">
         <is>
@@ -4694,7 +4694,7 @@
         <v>1</v>
       </c>
       <c r="Y37" t="n">
-        <v>0.01</v>
+        <v>0.05</v>
       </c>
       <c r="Z37" t="inlineStr">
         <is>
@@ -4809,7 +4809,7 @@
         <v>0.9572000000000001</v>
       </c>
       <c r="Y38" t="n">
-        <v>0.32</v>
+        <v>0.23</v>
       </c>
       <c r="Z38" t="inlineStr">
         <is>
@@ -4924,7 +4924,7 @@
         <v>0.994</v>
       </c>
       <c r="Y39" t="n">
-        <v>0.05</v>
+        <v>0.01</v>
       </c>
       <c r="Z39" t="inlineStr">
         <is>
@@ -5039,7 +5039,7 @@
         <v>1</v>
       </c>
       <c r="Y40" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.03</v>
       </c>
       <c r="Z40" t="inlineStr">
         <is>
@@ -5154,7 +5154,7 @@
         <v>0.9883999999999999</v>
       </c>
       <c r="Y41" t="n">
-        <v>0.15</v>
+        <v>0.2</v>
       </c>
       <c r="Z41" t="inlineStr">
         <is>
@@ -5269,7 +5269,7 @@
         <v>0.9196</v>
       </c>
       <c r="Y42" t="n">
-        <v>0.14</v>
+        <v>0.13</v>
       </c>
       <c r="Z42" t="inlineStr">
         <is>
@@ -5384,7 +5384,7 @@
         <v>0.8544</v>
       </c>
       <c r="Y43" t="n">
-        <v>0.33</v>
+        <v>0.19</v>
       </c>
       <c r="Z43" t="inlineStr">
         <is>
@@ -5499,7 +5499,7 @@
         <v>0.972</v>
       </c>
       <c r="Y44" t="n">
-        <v>0.26</v>
+        <v>0.15</v>
       </c>
       <c r="Z44" t="inlineStr">
         <is>
@@ -5614,7 +5614,7 @@
         <v>0.946</v>
       </c>
       <c r="Y45" t="n">
-        <v>0.4</v>
+        <v>0.24</v>
       </c>
       <c r="Z45" t="inlineStr">
         <is>
@@ -5729,7 +5729,7 @@
         <v>0.9565</v>
       </c>
       <c r="Y46" t="n">
-        <v>0.09</v>
+        <v>0.1</v>
       </c>
       <c r="Z46" t="inlineStr">
         <is>
@@ -5844,7 +5844,7 @@
         <v>0.9473</v>
       </c>
       <c r="Y47" t="n">
-        <v>0.2</v>
+        <v>0.21</v>
       </c>
       <c r="Z47" t="inlineStr">
         <is>
@@ -5959,7 +5959,7 @@
         <v>0.9496</v>
       </c>
       <c r="Y48" t="n">
-        <v>0.05</v>
+        <v>0.01</v>
       </c>
       <c r="Z48" t="inlineStr">
         <is>
@@ -6074,7 +6074,7 @@
         <v>0.9028</v>
       </c>
       <c r="Y49" t="n">
-        <v>0.16</v>
+        <v>0.13</v>
       </c>
       <c r="Z49" t="inlineStr">
         <is>
@@ -6189,7 +6189,7 @@
         <v>0.9031</v>
       </c>
       <c r="Y50" t="n">
-        <v>0.3</v>
+        <v>0.22</v>
       </c>
       <c r="Z50" t="inlineStr">
         <is>
@@ -6419,7 +6419,7 @@
         <v>0.97</v>
       </c>
       <c r="Y52" t="n">
-        <v>0.11</v>
+        <v>0.13</v>
       </c>
       <c r="Z52" t="inlineStr">
         <is>
@@ -6534,7 +6534,7 @@
         <v>0.9871</v>
       </c>
       <c r="Y53" t="n">
-        <v>0.16</v>
+        <v>0.15</v>
       </c>
       <c r="Z53" t="inlineStr">
         <is>
@@ -6649,7 +6649,7 @@
         <v>0.7585</v>
       </c>
       <c r="Y54" t="n">
-        <v>0.3</v>
+        <v>0.16</v>
       </c>
       <c r="Z54" t="inlineStr">
         <is>
@@ -6764,7 +6764,7 @@
         <v>0.9167</v>
       </c>
       <c r="Y55" t="n">
-        <v>0.18</v>
+        <v>0.15</v>
       </c>
       <c r="Z55" t="inlineStr">
         <is>
@@ -6879,7 +6879,7 @@
         <v>1</v>
       </c>
       <c r="Y56" t="n">
-        <v>0.08</v>
+        <v>0.06</v>
       </c>
       <c r="Z56" t="inlineStr">
         <is>
@@ -6994,7 +6994,7 @@
         <v>0.9859</v>
       </c>
       <c r="Y57" t="n">
-        <v>0.11</v>
+        <v>0.18</v>
       </c>
       <c r="Z57" t="inlineStr">
         <is>
@@ -7109,7 +7109,7 @@
         <v>0.9067</v>
       </c>
       <c r="Y58" t="n">
-        <v>0.25</v>
+        <v>0.24</v>
       </c>
       <c r="Z58" t="inlineStr">
         <is>
@@ -7224,7 +7224,7 @@
         <v>0.9869</v>
       </c>
       <c r="Y59" t="n">
-        <v>0.15</v>
+        <v>0.21</v>
       </c>
       <c r="Z59" t="inlineStr">
         <is>
@@ -7454,7 +7454,7 @@
         <v>1</v>
       </c>
       <c r="Y61" t="n">
-        <v>0.06</v>
+        <v>0.08</v>
       </c>
       <c r="Z61" t="inlineStr">
         <is>
@@ -7569,7 +7569,7 @@
         <v>0.9415</v>
       </c>
       <c r="Y62" t="n">
-        <v>0.12</v>
+        <v>0.17</v>
       </c>
       <c r="Z62" t="inlineStr">
         <is>
@@ -7684,7 +7684,7 @@
         <v>0.9391</v>
       </c>
       <c r="Y63" t="n">
-        <v>0.02</v>
+        <v>0</v>
       </c>
       <c r="Z63" t="inlineStr">
         <is>
@@ -7799,7 +7799,7 @@
         <v>0.851</v>
       </c>
       <c r="Y64" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="Z64" t="inlineStr">
         <is>
@@ -8029,7 +8029,7 @@
         <v>1</v>
       </c>
       <c r="Y66" t="n">
-        <v>0.08</v>
+        <v>0.09</v>
       </c>
       <c r="Z66" t="inlineStr">
         <is>
@@ -8259,7 +8259,7 @@
         <v>0.9297</v>
       </c>
       <c r="Y68" t="n">
-        <v>0.12</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="Z68" t="inlineStr">
         <is>
@@ -8374,7 +8374,7 @@
         <v>0.919</v>
       </c>
       <c r="Y69" t="n">
-        <v>0.24</v>
+        <v>0.25</v>
       </c>
       <c r="Z69" t="inlineStr">
         <is>
@@ -8489,7 +8489,7 @@
         <v>0.9693000000000001</v>
       </c>
       <c r="Y70" t="n">
-        <v>0.05</v>
+        <v>0.13</v>
       </c>
       <c r="Z70" t="inlineStr">
         <is>
@@ -8834,7 +8834,7 @@
         <v>1</v>
       </c>
       <c r="Y73" t="n">
-        <v>0.1</v>
+        <v>0.06</v>
       </c>
       <c r="Z73" t="inlineStr">
         <is>
@@ -8949,7 +8949,7 @@
         <v>0.9494</v>
       </c>
       <c r="Y74" t="n">
-        <v>0.06</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="Z74" t="inlineStr">
         <is>
@@ -9064,7 +9064,7 @@
         <v>1</v>
       </c>
       <c r="Y75" t="n">
-        <v>0.03</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="Z75" t="inlineStr">
         <is>
@@ -9294,7 +9294,7 @@
         <v>0.9368</v>
       </c>
       <c r="Y77" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.08</v>
       </c>
       <c r="Z77" t="inlineStr">
         <is>
@@ -9524,7 +9524,7 @@
         <v>1</v>
       </c>
       <c r="Y79" t="n">
-        <v>0.1</v>
+        <v>0.04</v>
       </c>
       <c r="Z79" t="inlineStr">
         <is>
@@ -9639,7 +9639,7 @@
         <v>0.9731</v>
       </c>
       <c r="Y80" t="n">
-        <v>0.02</v>
+        <v>0.04</v>
       </c>
       <c r="Z80" t="inlineStr">
         <is>
@@ -9869,7 +9869,7 @@
         <v>0.9784</v>
       </c>
       <c r="Y82" t="n">
-        <v>0.3</v>
+        <v>0.35</v>
       </c>
       <c r="Z82" t="inlineStr">
         <is>
@@ -10099,7 +10099,7 @@
         <v>0.864</v>
       </c>
       <c r="Y84" t="n">
-        <v>0.17</v>
+        <v>0.15</v>
       </c>
       <c r="Z84" t="inlineStr">
         <is>
@@ -10214,7 +10214,7 @@
         <v>0.9419999999999999</v>
       </c>
       <c r="Y85" t="n">
-        <v>0.01</v>
+        <v>0.03</v>
       </c>
       <c r="Z85" t="inlineStr">
         <is>
@@ -10329,7 +10329,7 @@
         <v>0.9104</v>
       </c>
       <c r="Y86" t="n">
-        <v>0.16</v>
+        <v>0.23</v>
       </c>
       <c r="Z86" t="inlineStr">
         <is>
@@ -10674,7 +10674,7 @@
         <v>0.8908</v>
       </c>
       <c r="Y89" t="n">
-        <v>0.13</v>
+        <v>0.18</v>
       </c>
       <c r="Z89" t="inlineStr">
         <is>
@@ -10789,7 +10789,7 @@
         <v>0.895</v>
       </c>
       <c r="Y90" t="n">
-        <v>0.24</v>
+        <v>0.32</v>
       </c>
       <c r="Z90" t="inlineStr">
         <is>
@@ -10904,7 +10904,7 @@
         <v>1</v>
       </c>
       <c r="Y91" t="n">
-        <v>0.05</v>
+        <v>0.06</v>
       </c>
       <c r="Z91" t="inlineStr">
         <is>
@@ -11019,7 +11019,7 @@
         <v>1</v>
       </c>
       <c r="Y92" t="n">
-        <v>0.08</v>
+        <v>0.13</v>
       </c>
       <c r="Z92" t="inlineStr">
         <is>
@@ -11134,7 +11134,7 @@
         <v>1</v>
       </c>
       <c r="Y93" t="n">
-        <v>0.05</v>
+        <v>0.01</v>
       </c>
       <c r="Z93" t="inlineStr">
         <is>
@@ -11249,7 +11249,7 @@
         <v>0.9703000000000001</v>
       </c>
       <c r="Y94" t="n">
-        <v>0.06</v>
+        <v>0.1</v>
       </c>
       <c r="Z94" t="inlineStr">
         <is>
@@ -11479,7 +11479,7 @@
         <v>0.9699</v>
       </c>
       <c r="Y96" t="n">
-        <v>0.13</v>
+        <v>0.16</v>
       </c>
       <c r="Z96" t="inlineStr">
         <is>
@@ -11824,7 +11824,7 @@
         <v>0.9824000000000001</v>
       </c>
       <c r="Y99" t="n">
-        <v>0.12</v>
+        <v>0.02</v>
       </c>
       <c r="Z99" t="inlineStr">
         <is>
@@ -11939,7 +11939,7 @@
         <v>0.9516</v>
       </c>
       <c r="Y100" t="n">
-        <v>0.08</v>
+        <v>0.05</v>
       </c>
       <c r="Z100" t="inlineStr">
         <is>
@@ -12054,7 +12054,7 @@
         <v>0.9034</v>
       </c>
       <c r="Y101" t="n">
-        <v>0.17</v>
+        <v>0.16</v>
       </c>
       <c r="Z101" t="inlineStr">
         <is>
@@ -12169,7 +12169,7 @@
         <v>1</v>
       </c>
       <c r="Y102" t="n">
-        <v>0.01</v>
+        <v>0.03</v>
       </c>
       <c r="Z102" t="inlineStr">
         <is>
@@ -12284,7 +12284,7 @@
         <v>0.9554</v>
       </c>
       <c r="Y103" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.12</v>
       </c>
       <c r="Z103" t="inlineStr">
         <is>
@@ -12514,7 +12514,7 @@
         <v>0.9035</v>
       </c>
       <c r="Y105" t="n">
-        <v>0.01</v>
+        <v>0.02</v>
       </c>
       <c r="Z105" t="inlineStr">
         <is>
@@ -12629,7 +12629,7 @@
         <v>0.8697</v>
       </c>
       <c r="Y106" t="n">
-        <v>0.2</v>
+        <v>0.26</v>
       </c>
       <c r="Z106" t="inlineStr">
         <is>
@@ -12744,7 +12744,7 @@
         <v>0.8582</v>
       </c>
       <c r="Y107" t="n">
-        <v>0.05</v>
+        <v>0.08</v>
       </c>
       <c r="Z107" t="inlineStr">
         <is>
@@ -13089,7 +13089,7 @@
         <v>1</v>
       </c>
       <c r="Y110" t="n">
-        <v>0.08</v>
+        <v>0.12</v>
       </c>
       <c r="Z110" t="inlineStr">
         <is>
@@ -13204,7 +13204,7 @@
         <v>1</v>
       </c>
       <c r="Y111" t="n">
-        <v>0.04</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="Z111" t="inlineStr">
         <is>
@@ -13319,7 +13319,7 @@
         <v>0.9801</v>
       </c>
       <c r="Y112" t="n">
-        <v>0.16</v>
+        <v>0.1</v>
       </c>
       <c r="Z112" t="inlineStr">
         <is>
@@ -13664,7 +13664,7 @@
         <v>0.9848</v>
       </c>
       <c r="Y115" t="n">
-        <v>0.24</v>
+        <v>0.28</v>
       </c>
       <c r="Z115" t="inlineStr">
         <is>
@@ -13779,7 +13779,7 @@
         <v>0.9678</v>
       </c>
       <c r="Y116" t="n">
-        <v>0.26</v>
+        <v>0.25</v>
       </c>
       <c r="Z116" t="inlineStr">
         <is>
@@ -14124,7 +14124,7 @@
         <v>1</v>
       </c>
       <c r="Y119" t="n">
-        <v>0.02</v>
+        <v>0.01</v>
       </c>
       <c r="Z119" t="inlineStr">
         <is>
@@ -14239,7 +14239,7 @@
         <v>1</v>
       </c>
       <c r="Y120" t="n">
-        <v>0.04</v>
+        <v>0.03</v>
       </c>
       <c r="Z120" t="inlineStr">
         <is>
@@ -14469,7 +14469,7 @@
         <v>0.895</v>
       </c>
       <c r="Y122" t="n">
-        <v>0.21</v>
+        <v>0.17</v>
       </c>
       <c r="Z122" t="inlineStr">
         <is>
@@ -14584,7 +14584,7 @@
         <v>0.9533</v>
       </c>
       <c r="Y123" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.04</v>
       </c>
       <c r="Z123" t="inlineStr">
         <is>
@@ -14699,7 +14699,7 @@
         <v>0.9696</v>
       </c>
       <c r="Y124" t="n">
-        <v>0.04</v>
+        <v>0.03</v>
       </c>
       <c r="Z124" t="inlineStr">
         <is>
@@ -14929,7 +14929,7 @@
         <v>0.9523</v>
       </c>
       <c r="Y126" t="n">
-        <v>0.12</v>
+        <v>0.14</v>
       </c>
       <c r="Z126" t="inlineStr">
         <is>
@@ -15274,7 +15274,7 @@
         <v>0.9919</v>
       </c>
       <c r="Y129" t="n">
-        <v>0.04</v>
+        <v>0.03</v>
       </c>
       <c r="Z129" t="inlineStr">
         <is>
@@ -15389,7 +15389,7 @@
         <v>1</v>
       </c>
       <c r="Y130" t="n">
-        <v>0.01</v>
+        <v>0</v>
       </c>
       <c r="Z130" t="inlineStr">
         <is>
@@ -15504,7 +15504,7 @@
         <v>0.9785</v>
       </c>
       <c r="Y131" t="n">
-        <v>0.13</v>
+        <v>0.1</v>
       </c>
       <c r="Z131" t="inlineStr">
         <is>
@@ -15619,7 +15619,7 @@
         <v>0.954</v>
       </c>
       <c r="Y132" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.02</v>
       </c>
       <c r="Z132" t="inlineStr">
         <is>
@@ -15734,7 +15734,7 @@
         <v>0.9354</v>
       </c>
       <c r="Y133" t="n">
-        <v>0.08</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="Z133" t="inlineStr">
         <is>
@@ -15849,7 +15849,7 @@
         <v>1</v>
       </c>
       <c r="Y134" t="n">
-        <v>0.03</v>
+        <v>0.01</v>
       </c>
       <c r="Z134" t="inlineStr">
         <is>
@@ -15964,7 +15964,7 @@
         <v>0.9414</v>
       </c>
       <c r="Y135" t="n">
-        <v>0.01</v>
+        <v>0.02</v>
       </c>
       <c r="Z135" t="inlineStr">
         <is>
@@ -16079,7 +16079,7 @@
         <v>1</v>
       </c>
       <c r="Y136" t="n">
-        <v>0.09</v>
+        <v>0.02</v>
       </c>
       <c r="Z136" t="inlineStr">
         <is>
@@ -16194,7 +16194,7 @@
         <v>0.9694</v>
       </c>
       <c r="Y137" t="n">
-        <v>0.18</v>
+        <v>0.08</v>
       </c>
       <c r="Z137" t="inlineStr">
         <is>
@@ -16309,7 +16309,7 @@
         <v>0.8774</v>
       </c>
       <c r="Y138" t="n">
-        <v>0.12</v>
+        <v>0.1</v>
       </c>
       <c r="Z138" t="inlineStr">
         <is>
@@ -16424,7 +16424,7 @@
         <v>0.9896</v>
       </c>
       <c r="Y139" t="n">
-        <v>0.32</v>
+        <v>0.2</v>
       </c>
       <c r="Z139" t="inlineStr">
         <is>
@@ -16539,7 +16539,7 @@
         <v>1</v>
       </c>
       <c r="Y140" t="n">
-        <v>0.02</v>
+        <v>0.01</v>
       </c>
       <c r="Z140" t="inlineStr">
         <is>
@@ -16884,7 +16884,7 @@
         <v>0.9796</v>
       </c>
       <c r="Y143" t="n">
-        <v>0.08</v>
+        <v>0.12</v>
       </c>
       <c r="Z143" t="inlineStr">
         <is>
@@ -16999,7 +16999,7 @@
         <v>1</v>
       </c>
       <c r="Y144" t="n">
-        <v>0.05</v>
+        <v>0.03</v>
       </c>
       <c r="Z144" t="inlineStr">
         <is>
@@ -17229,7 +17229,7 @@
         <v>1</v>
       </c>
       <c r="Y146" t="n">
-        <v>0.04</v>
+        <v>0.02</v>
       </c>
       <c r="Z146" t="inlineStr">
         <is>
@@ -17344,7 +17344,7 @@
         <v>0.983</v>
       </c>
       <c r="Y147" t="n">
-        <v>0.17</v>
+        <v>0.18</v>
       </c>
       <c r="Z147" t="inlineStr">
         <is>
@@ -17459,7 +17459,7 @@
         <v>1</v>
       </c>
       <c r="Y148" t="n">
-        <v>0.05</v>
+        <v>0.04</v>
       </c>
       <c r="Z148" t="inlineStr">
         <is>
@@ -17574,7 +17574,7 @@
         <v>0.99</v>
       </c>
       <c r="Y149" t="n">
-        <v>0.08</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="Z149" t="inlineStr">
         <is>
@@ -17689,7 +17689,7 @@
         <v>1</v>
       </c>
       <c r="Y150" t="n">
-        <v>0.1</v>
+        <v>0.05</v>
       </c>
       <c r="Z150" t="inlineStr">
         <is>
@@ -17804,7 +17804,7 @@
         <v>0.9796</v>
       </c>
       <c r="Y151" t="n">
-        <v>0.19</v>
+        <v>0.17</v>
       </c>
       <c r="Z151" t="inlineStr">
         <is>
@@ -17919,7 +17919,7 @@
         <v>0.9752999999999999</v>
       </c>
       <c r="Y152" t="n">
-        <v>0.04</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="Z152" t="inlineStr">
         <is>
@@ -18034,7 +18034,7 @@
         <v>1</v>
       </c>
       <c r="Y153" t="n">
-        <v>0.02</v>
+        <v>0.01</v>
       </c>
       <c r="Z153" t="inlineStr">
         <is>
@@ -18149,7 +18149,7 @@
         <v>0.8913</v>
       </c>
       <c r="Y154" t="n">
-        <v>0.25</v>
+        <v>0.23</v>
       </c>
       <c r="Z154" t="inlineStr">
         <is>
@@ -18264,7 +18264,7 @@
         <v>0.9288999999999999</v>
       </c>
       <c r="Y155" t="n">
-        <v>0.16</v>
+        <v>0.13</v>
       </c>
       <c r="Z155" t="inlineStr">
         <is>
@@ -18494,7 +18494,7 @@
         <v>0.9396</v>
       </c>
       <c r="Y157" t="n">
-        <v>0.18</v>
+        <v>0.06</v>
       </c>
       <c r="Z157" t="inlineStr">
         <is>
@@ -18609,7 +18609,7 @@
         <v>1</v>
       </c>
       <c r="Y158" t="n">
-        <v>0.03</v>
+        <v>0.01</v>
       </c>
       <c r="Z158" t="inlineStr">
         <is>
@@ -18724,7 +18724,7 @@
         <v>0.9529</v>
       </c>
       <c r="Y159" t="n">
-        <v>0.14</v>
+        <v>0.11</v>
       </c>
       <c r="Z159" t="inlineStr">
         <is>
@@ -18839,7 +18839,7 @@
         <v>1</v>
       </c>
       <c r="Y160" t="n">
-        <v>0.12</v>
+        <v>0.05</v>
       </c>
       <c r="Z160" t="inlineStr">
         <is>
@@ -18954,7 +18954,7 @@
         <v>0.9746</v>
       </c>
       <c r="Y161" t="n">
-        <v>0.06</v>
+        <v>0.05</v>
       </c>
       <c r="Z161" t="inlineStr">
         <is>
@@ -19069,7 +19069,7 @@
         <v>0.9963</v>
       </c>
       <c r="Y162" t="n">
-        <v>0.06</v>
+        <v>0.09</v>
       </c>
       <c r="Z162" t="inlineStr">
         <is>
@@ -19184,11 +19184,11 @@
         <v>0.893</v>
       </c>
       <c r="Y163" t="n">
-        <v>0.36</v>
+        <v>0.41</v>
       </c>
       <c r="Z163" t="inlineStr">
         <is>
-          <t>NO (Pruned)</t>
+          <t>YES (Collided)</t>
         </is>
       </c>
       <c r="AA163" t="inlineStr">
@@ -19414,7 +19414,7 @@
         <v>0.9594</v>
       </c>
       <c r="Y165" t="n">
-        <v>0.16</v>
+        <v>0.17</v>
       </c>
       <c r="Z165" t="inlineStr">
         <is>
@@ -19529,7 +19529,7 @@
         <v>1</v>
       </c>
       <c r="Y166" t="n">
-        <v>0</v>
+        <v>0.04</v>
       </c>
       <c r="Z166" t="inlineStr">
         <is>
@@ -19644,7 +19644,7 @@
         <v>0.9528</v>
       </c>
       <c r="Y167" t="n">
-        <v>0.23</v>
+        <v>0.15</v>
       </c>
       <c r="Z167" t="inlineStr">
         <is>
@@ -19759,7 +19759,7 @@
         <v>0.9532</v>
       </c>
       <c r="Y168" t="n">
-        <v>0.22</v>
+        <v>0.29</v>
       </c>
       <c r="Z168" t="inlineStr">
         <is>
@@ -19874,7 +19874,7 @@
         <v>0.981</v>
       </c>
       <c r="Y169" t="n">
-        <v>0.05</v>
+        <v>0.03</v>
       </c>
       <c r="Z169" t="inlineStr">
         <is>
@@ -20104,7 +20104,7 @@
         <v>0.9718</v>
       </c>
       <c r="Y171" t="n">
-        <v>0.09</v>
+        <v>0.08</v>
       </c>
       <c r="Z171" t="inlineStr">
         <is>
@@ -20219,7 +20219,7 @@
         <v>0.977</v>
       </c>
       <c r="Y172" t="n">
-        <v>0.13</v>
+        <v>0.17</v>
       </c>
       <c r="Z172" t="inlineStr">
         <is>
@@ -20449,7 +20449,7 @@
         <v>0.9659</v>
       </c>
       <c r="Y174" t="n">
-        <v>0.18</v>
+        <v>0.16</v>
       </c>
       <c r="Z174" t="inlineStr">
         <is>
@@ -20564,7 +20564,7 @@
         <v>0.6267</v>
       </c>
       <c r="Y175" t="n">
-        <v>0.39</v>
+        <v>0.44</v>
       </c>
       <c r="Z175" t="inlineStr">
         <is>
@@ -20679,7 +20679,7 @@
         <v>0.9816</v>
       </c>
       <c r="Y176" t="n">
-        <v>0.13</v>
+        <v>0.15</v>
       </c>
       <c r="Z176" t="inlineStr">
         <is>
@@ -20909,7 +20909,7 @@
         <v>1</v>
       </c>
       <c r="Y178" t="n">
-        <v>0.05</v>
+        <v>0.01</v>
       </c>
       <c r="Z178" t="inlineStr">
         <is>
@@ -21024,7 +21024,7 @@
         <v>0.9826</v>
       </c>
       <c r="Y179" t="n">
-        <v>0.05</v>
+        <v>0.04</v>
       </c>
       <c r="Z179" t="inlineStr">
         <is>
@@ -21139,7 +21139,7 @@
         <v>1</v>
       </c>
       <c r="Y180" t="n">
-        <v>0.05</v>
+        <v>0.1</v>
       </c>
       <c r="Z180" t="inlineStr">
         <is>
@@ -21254,7 +21254,7 @@
         <v>1</v>
       </c>
       <c r="Y181" t="n">
-        <v>0.14</v>
+        <v>0.11</v>
       </c>
       <c r="Z181" t="inlineStr">
         <is>
@@ -21369,7 +21369,7 @@
         <v>0.9881</v>
       </c>
       <c r="Y182" t="n">
-        <v>0.16</v>
+        <v>0.25</v>
       </c>
       <c r="Z182" t="inlineStr">
         <is>
@@ -21484,7 +21484,7 @@
         <v>1</v>
       </c>
       <c r="Y183" t="n">
-        <v>0.03</v>
+        <v>0.06</v>
       </c>
       <c r="Z183" t="inlineStr">
         <is>
@@ -21599,7 +21599,7 @@
         <v>0.8469</v>
       </c>
       <c r="Y184" t="n">
-        <v>0.27</v>
+        <v>0.33</v>
       </c>
       <c r="Z184" t="inlineStr">
         <is>

</xml_diff>